<commit_message>
Update plan and excel files
</commit_message>
<xml_diff>
--- a/Check.xlsx
+++ b/Check.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="53">
   <si>
     <t xml:space="preserve">    Функционал</t>
   </si>
@@ -19,7 +19,10 @@
     <t xml:space="preserve">                            Проверка</t>
   </si>
   <si>
-    <t xml:space="preserve">   Результат</t>
+    <t xml:space="preserve">   Приоритет</t>
+  </si>
+  <si>
+    <t>Результат</t>
   </si>
   <si>
     <t>Авторизация</t>
@@ -28,12 +31,30 @@
     <t>Вход с валидными данными (login2/password2)</t>
   </si>
   <si>
-    <t xml:space="preserve">	Пройдено</t>
+    <t xml:space="preserve">        High</t>
+  </si>
+  <si>
+    <t>Pass</t>
   </si>
   <si>
     <t xml:space="preserve">	Попытка входа с пустыми полями</t>
   </si>
   <si>
+    <t xml:space="preserve">	Ввод неверного пароля</t>
+  </si>
+  <si>
+    <t>Ввод логина в разном регистре</t>
+  </si>
+  <si>
+    <t xml:space="preserve">       Medium</t>
+  </si>
+  <si>
+    <t>Скрытие символов в поле «Пароль»</t>
+  </si>
+  <si>
+    <t xml:space="preserve">      Medium</t>
+  </si>
+  <si>
     <t>Новости</t>
   </si>
   <si>
@@ -43,7 +64,22 @@
     <t xml:space="preserve">	Разворачивание описания новости по клику</t>
   </si>
   <si>
-    <t xml:space="preserve">        	Фильтрация новостей по категории</t>
+    <t>Сворачивание описания новости</t>
+  </si>
+  <si>
+    <t>Фильтрация новостей по категории «Объявление»</t>
+  </si>
+  <si>
+    <t>Фильтрация новостей по категории «День рождения»</t>
+  </si>
+  <si>
+    <t>Работа фильтра «от даты до даты»</t>
+  </si>
+  <si>
+    <t>Обновление списка (Pull-to-refresh)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         Low</t>
   </si>
   <si>
     <t>Control Panel</t>
@@ -55,23 +91,92 @@
     <t xml:space="preserve">	Создание новой новости (кнопка "+")</t>
   </si>
   <si>
+    <t>Редактирование заголовка существующей новости</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        High  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">	Удаление новости через иконку корзины</t>
+  </si>
+  <si>
+    <t>Отмена удаления новости в диалоговом окне</t>
+  </si>
+  <si>
+    <t>Создание новости с очень длинным заголовком</t>
+  </si>
+  <si>
+    <t>Создание новости без выбора даты</t>
+  </si>
+  <si>
     <t>Цитаты</t>
   </si>
   <si>
     <t xml:space="preserve">	Переход в раздел "Our Mission" (бабочка)</t>
   </si>
   <si>
+    <t>Прокрутка (Scroll) списка цитат</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
     <t>О приложении</t>
   </si>
   <si>
     <t>Переход в раздел "About"</t>
+  </si>
+  <si>
+    <t>Наличие ссылки на политику конфиденциальности</t>
+  </si>
+  <si>
+    <t>UI/UX</t>
+  </si>
+  <si>
+    <t>Наличие иконки приложения в меню телефона</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     Medium</t>
+  </si>
+  <si>
+    <t>Кликабельность всех элементов верхнего меню</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>Нефункционал</t>
+  </si>
+  <si>
+    <t>Смена ориентации экрана (верт./гориз.)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        Medium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">	Работа приложения при выключенном интернете</t>
+  </si>
+  <si>
+    <t>Fail</t>
+  </si>
+  <si>
+    <t>Сворачивание приложения при входящем звонке</t>
+  </si>
+  <si>
+    <t>Возврат в приложение из фонового режима</t>
+  </si>
+  <si>
+    <t>Корректность верстки на малом экране (эмулятор)</t>
+  </si>
+  <si>
+    <t>Скорость загрузки новостей (менее 3 секунд)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -80,6 +185,13 @@
     </font>
     <font>
       <b/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10.0"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
@@ -104,18 +216,33 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="9">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="center"/>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -346,146 +473,447 @@
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="2" t="s">
+      <c r="A2" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="B2" s="4" t="s">
         <v>5</v>
       </c>
+      <c r="C2" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="2" t="s">
+      <c r="A3" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>5</v>
+      <c r="D3" s="6" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>5</v>
+      <c r="A4" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>5</v>
+      <c r="A5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>5</v>
+      <c r="A6" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="s">
+      <c r="D9" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C11" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="D11" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="E16" s="8"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C18" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C10" s="3"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="3"/>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="3"/>
-      <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="3"/>
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="3"/>
-      <c r="B14" s="3"/>
-      <c r="C14" s="3"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="3"/>
-      <c r="B15" s="3"/>
-      <c r="C15" s="3"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="3"/>
-      <c r="B16" s="3"/>
-      <c r="C16" s="3"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="3"/>
-      <c r="B17" s="3"/>
-      <c r="C17" s="3"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="3"/>
-      <c r="B18" s="3"/>
-      <c r="C18" s="3"/>
+      <c r="D18" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="D22" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="24" ht="33.0" customHeight="1">
+      <c r="A24" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="D24" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="D25" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="D27" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D28" s="6" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="D29" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="D30" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="D31" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="D32" s="6" t="s">
+        <v>7</v>
+      </c>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>

</xml_diff>